<commit_message>
Add sourcing updates and unify procedure data access
</commit_message>
<xml_diff>
--- a/Manual_Extraction_Index.xlsx
+++ b/Manual_Extraction_Index.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L229"/>
+  <dimension ref="A1:L317"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10392,16 +10392,32 @@
     </row>
     <row r="226">
       <c r="A226" t="inlineStr"/>
-      <c r="B226" t="inlineStr"/>
-      <c r="C226" t="inlineStr"/>
-      <c r="D226" t="inlineStr"/>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Acumed Elbow arthroplasty Portfolio</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>portfolio_page</t>
+        </is>
+      </c>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Acumed Elbow Arthroplasty Portfolio</t>
+        </is>
+      </c>
       <c r="E226" t="inlineStr"/>
-      <c r="F226" t="inlineStr"/>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
       <c r="G226" t="n">
         <v>0</v>
       </c>
       <c r="H226" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I226" t="n">
         <v>0</v>
@@ -10410,93 +10426,4053 @@
         <v>0</v>
       </c>
       <c r="K226" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L226" t="inlineStr">
         <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_ACUMED_ELBOW_ARTHROPLASTY_PORTFOLIO_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Acute Care Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>society_about_page</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>AAST Acute Care Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr"/>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G227" t="n">
+        <v>0</v>
+      </c>
+      <c r="H227" t="n">
+        <v>1</v>
+      </c>
+      <c r="I227" t="n">
+        <v>0</v>
+      </c>
+      <c r="J227" t="n">
+        <v>0</v>
+      </c>
+      <c r="K227" t="n">
+        <v>2</v>
+      </c>
+      <c r="L227" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_ACUTE_CARE_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Anaesthesia Information Management System</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>guidance_page</t>
+        </is>
+      </c>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>AIMS Overview / OpenAnesthesia</t>
+        </is>
+      </c>
+      <c r="E228" t="inlineStr"/>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G228" t="n">
+        <v>0</v>
+      </c>
+      <c r="H228" t="n">
+        <v>1</v>
+      </c>
+      <c r="I228" t="n">
+        <v>0</v>
+      </c>
+      <c r="J228" t="n">
+        <v>0</v>
+      </c>
+      <c r="K228" t="n">
+        <v>2</v>
+      </c>
+      <c r="L228" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_ANAESTHESIA_INFORMATION_MANAGEMENT_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>BD</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Arterial Line Kit</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>product_family_page</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>StatLock Arterial Ultra Stabilisation Device | BD</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr"/>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G229" t="n">
+        <v>0</v>
+      </c>
+      <c r="H229" t="n">
+        <v>2</v>
+      </c>
+      <c r="I229" t="n">
+        <v>1</v>
+      </c>
+      <c r="J229" t="n">
+        <v>0</v>
+      </c>
+      <c r="K229" t="n">
+        <v>1</v>
+      </c>
+      <c r="L229" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_ARTERIAL_LINE_KIT_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Bariatric Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>ASMBS / IFSO Bariatric Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr"/>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G230" t="n">
+        <v>0</v>
+      </c>
+      <c r="H230" t="n">
+        <v>1</v>
+      </c>
+      <c r="I230" t="n">
+        <v>0</v>
+      </c>
+      <c r="J230" t="n">
+        <v>0</v>
+      </c>
+      <c r="K230" t="n">
+        <v>2</v>
+      </c>
+      <c r="L230" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_BARIATRIC_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr"/>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Breast Reconstruction Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>BAPRAS / ASPS Breast Reconstruction Resources</t>
+        </is>
+      </c>
+      <c r="E231" t="inlineStr"/>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G231" t="n">
+        <v>0</v>
+      </c>
+      <c r="H231" t="n">
+        <v>1</v>
+      </c>
+      <c r="I231" t="n">
+        <v>0</v>
+      </c>
+      <c r="J231" t="n">
+        <v>0</v>
+      </c>
+      <c r="K231" t="n">
+        <v>2</v>
+      </c>
+      <c r="L231" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_BREAST_RECONSTRUCTION_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Breast Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>ASBrS / ABS Breast Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr"/>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G232" t="n">
+        <v>0</v>
+      </c>
+      <c r="H232" t="n">
+        <v>1</v>
+      </c>
+      <c r="I232" t="n">
+        <v>0</v>
+      </c>
+      <c r="J232" t="n">
+        <v>0</v>
+      </c>
+      <c r="K232" t="n">
+        <v>2</v>
+      </c>
+      <c r="L232" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_BREAST_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr"/>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Burns Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>BAPRAS / ABA Burns Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr"/>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G233" t="n">
+        <v>0</v>
+      </c>
+      <c r="H233" t="n">
+        <v>1</v>
+      </c>
+      <c r="I233" t="n">
+        <v>0</v>
+      </c>
+      <c r="J233" t="n">
+        <v>0</v>
+      </c>
+      <c r="K233" t="n">
+        <v>2</v>
+      </c>
+      <c r="L233" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_BURNS_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr"/>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Caesarean Birth Information System</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>RCOG / ACOG Caesarean Birth Resources</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr"/>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G234" t="n">
+        <v>0</v>
+      </c>
+      <c r="H234" t="n">
+        <v>1</v>
+      </c>
+      <c r="I234" t="n">
+        <v>0</v>
+      </c>
+      <c r="J234" t="n">
+        <v>0</v>
+      </c>
+      <c r="K234" t="n">
+        <v>2</v>
+      </c>
+      <c r="L234" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_CAESAREAN_BIRTH_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Cardiac Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>society_about_page</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>STS / EACTS Cardiac Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E235" t="inlineStr"/>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G235" t="n">
+        <v>0</v>
+      </c>
+      <c r="H235" t="n">
+        <v>1</v>
+      </c>
+      <c r="I235" t="n">
+        <v>0</v>
+      </c>
+      <c r="J235" t="n">
+        <v>0</v>
+      </c>
+      <c r="K235" t="n">
+        <v>2</v>
+      </c>
+      <c r="L235" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_CARDIAC_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Cardiothoracic Anaesthesia Workflow System</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>practice_resources</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>SCA Practice Resources / E-Manual of Cardiac Anesthesia</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr"/>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G236" t="n">
+        <v>0</v>
+      </c>
+      <c r="H236" t="n">
+        <v>1</v>
+      </c>
+      <c r="I236" t="n">
+        <v>0</v>
+      </c>
+      <c r="J236" t="n">
+        <v>0</v>
+      </c>
+      <c r="K236" t="n">
+        <v>2</v>
+      </c>
+      <c r="L236" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_CARDIOTHORACIC_ANAESTHESIA_WORKFLOW_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr"/>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Cataract Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>RCOphth / ASCRS Cataract Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr"/>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G237" t="n">
+        <v>0</v>
+      </c>
+      <c r="H237" t="n">
+        <v>1</v>
+      </c>
+      <c r="I237" t="n">
+        <v>0</v>
+      </c>
+      <c r="J237" t="n">
+        <v>0</v>
+      </c>
+      <c r="K237" t="n">
+        <v>2</v>
+      </c>
+      <c r="L237" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_CATARACT_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr"/>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Cleft Lip and Palate Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>BAPRAS / ACPA Cleft Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E238" t="inlineStr"/>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G238" t="n">
+        <v>0</v>
+      </c>
+      <c r="H238" t="n">
+        <v>1</v>
+      </c>
+      <c r="I238" t="n">
+        <v>0</v>
+      </c>
+      <c r="J238" t="n">
+        <v>0</v>
+      </c>
+      <c r="K238" t="n">
+        <v>2</v>
+      </c>
+      <c r="L238" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_CLEFT_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Colorectal Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>ASCRS / ESCP Colorectal Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr"/>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G239" t="n">
+        <v>0</v>
+      </c>
+      <c r="H239" t="n">
+        <v>1</v>
+      </c>
+      <c r="I239" t="n">
+        <v>0</v>
+      </c>
+      <c r="J239" t="n">
+        <v>0</v>
+      </c>
+      <c r="K239" t="n">
+        <v>2</v>
+      </c>
+      <c r="L239" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_COLORECTAL_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Congenital Cardiac Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>database_page</t>
+        </is>
+      </c>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>STS CHSD / CHSS Resources</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr"/>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G240" t="n">
+        <v>0</v>
+      </c>
+      <c r="H240" t="n">
+        <v>1</v>
+      </c>
+      <c r="I240" t="n">
+        <v>0</v>
+      </c>
+      <c r="J240" t="n">
+        <v>0</v>
+      </c>
+      <c r="K240" t="n">
+        <v>2</v>
+      </c>
+      <c r="L240" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_CONGENITAL_CARDIAC_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr"/>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Corin Hip revision arthroplasty Portfolio</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>portfolio_page</t>
+        </is>
+      </c>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Corin Revision Hip Arthroplasty Portfolio</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr"/>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G241" t="n">
+        <v>0</v>
+      </c>
+      <c r="H241" t="n">
+        <v>1</v>
+      </c>
+      <c r="I241" t="n">
+        <v>0</v>
+      </c>
+      <c r="J241" t="n">
+        <v>0</v>
+      </c>
+      <c r="K241" t="n">
+        <v>2</v>
+      </c>
+      <c r="L241" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_CORIN_HIP_REVISION_ARTHROPLASTY_PORTFOLIO_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr"/>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Corneal and Anterior Segment Information System</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>RCOphth / ASCRS Corneal and Anterior Segment Resources</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr"/>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G242" t="n">
+        <v>0</v>
+      </c>
+      <c r="H242" t="n">
+        <v>1</v>
+      </c>
+      <c r="I242" t="n">
+        <v>0</v>
+      </c>
+      <c r="J242" t="n">
+        <v>0</v>
+      </c>
+      <c r="K242" t="n">
+        <v>2</v>
+      </c>
+      <c r="L242" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_CORNEAL_ANTERIOR_SEGMENT_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr"/>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Cranial Neurosurgery Information System</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>CNS / EANS Cranial Neurosurgery Resources</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr"/>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G243" t="n">
+        <v>0</v>
+      </c>
+      <c r="H243" t="n">
+        <v>1</v>
+      </c>
+      <c r="I243" t="n">
+        <v>0</v>
+      </c>
+      <c r="J243" t="n">
+        <v>0</v>
+      </c>
+      <c r="K243" t="n">
+        <v>2</v>
+      </c>
+      <c r="L243" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_CRANIAL_NEUROSURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr"/>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Craniofacial Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>BAPRAS / ISCFS Craniofacial Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr"/>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G244" t="n">
+        <v>0</v>
+      </c>
+      <c r="H244" t="n">
+        <v>1</v>
+      </c>
+      <c r="I244" t="n">
+        <v>0</v>
+      </c>
+      <c r="J244" t="n">
+        <v>0</v>
+      </c>
+      <c r="K244" t="n">
+        <v>2</v>
+      </c>
+      <c r="L244" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_CRANIOFACIAL_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>B. Braun</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Combined Spinal Epidural Kit</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>product_family_page</t>
+        </is>
+      </c>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Combined Spinal Epidural Trays (Kits)</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr"/>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G245" t="n">
+        <v>1</v>
+      </c>
+      <c r="H245" t="n">
+        <v>3</v>
+      </c>
+      <c r="I245" t="n">
+        <v>3</v>
+      </c>
+      <c r="J245" t="n">
+        <v>0</v>
+      </c>
+      <c r="K245" t="n">
+        <v>0</v>
+      </c>
+      <c r="L245" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_CSE_KIT_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>Teleflex</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Central Venous Catheter Kit</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>product_family_page</t>
+        </is>
+      </c>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>Central Access / Arrow ErgoPack Complete System | Teleflex</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr"/>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G246" t="n">
+        <v>1</v>
+      </c>
+      <c r="H246" t="n">
+        <v>3</v>
+      </c>
+      <c r="I246" t="n">
+        <v>1</v>
+      </c>
+      <c r="J246" t="n">
+        <v>0</v>
+      </c>
+      <c r="K246" t="n">
+        <v>1</v>
+      </c>
+      <c r="L246" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_CVC_KIT_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Dental Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>society_about_page</t>
+        </is>
+      </c>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>AAOMS / BAOMS Oral and Maxillofacial Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr"/>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G247" t="n">
+        <v>0</v>
+      </c>
+      <c r="H247" t="n">
+        <v>1</v>
+      </c>
+      <c r="I247" t="n">
+        <v>0</v>
+      </c>
+      <c r="J247" t="n">
+        <v>0</v>
+      </c>
+      <c r="K247" t="n">
+        <v>2</v>
+      </c>
+      <c r="L247" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_DENTAL_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr"/>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Dentoalveolar Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>BAOS / AAOMS Dentoalveolar Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr"/>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G248" t="n">
+        <v>0</v>
+      </c>
+      <c r="H248" t="n">
+        <v>1</v>
+      </c>
+      <c r="I248" t="n">
+        <v>0</v>
+      </c>
+      <c r="J248" t="n">
+        <v>0</v>
+      </c>
+      <c r="K248" t="n">
+        <v>2</v>
+      </c>
+      <c r="L248" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_DENTOALVEOLAR_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr"/>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>DePuy Synthes Elbow arthroplasty Portfolio</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>portfolio_page</t>
+        </is>
+      </c>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>DePuy Synthes Elbow Arthroplasty Portfolio</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr"/>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G249" t="n">
+        <v>0</v>
+      </c>
+      <c r="H249" t="n">
+        <v>1</v>
+      </c>
+      <c r="I249" t="n">
+        <v>0</v>
+      </c>
+      <c r="J249" t="n">
+        <v>0</v>
+      </c>
+      <c r="K249" t="n">
+        <v>2</v>
+      </c>
+      <c r="L249" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_DEPUY_SYNTHES_ELBOW_ARTHROPLASTY_PORTFOLIO_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr"/>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>DePuy Synthes Hip revision arthroplasty Portfolio</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>portfolio_page</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>DePuy Synthes Revision Hip Arthroplasty Portfolio</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr"/>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G250" t="n">
+        <v>0</v>
+      </c>
+      <c r="H250" t="n">
+        <v>1</v>
+      </c>
+      <c r="I250" t="n">
+        <v>0</v>
+      </c>
+      <c r="J250" t="n">
+        <v>0</v>
+      </c>
+      <c r="K250" t="n">
+        <v>2</v>
+      </c>
+      <c r="L250" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_DEPUY_SYNTHES_HIP_REVISION_ARTHROPLASTY_PORTFOLIO_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr"/>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Dermatologic Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>BSDS / ASDS Dermatologic Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr"/>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G251" t="n">
+        <v>0</v>
+      </c>
+      <c r="H251" t="n">
+        <v>1</v>
+      </c>
+      <c r="I251" t="n">
+        <v>0</v>
+      </c>
+      <c r="J251" t="n">
+        <v>0</v>
+      </c>
+      <c r="K251" t="n">
+        <v>2</v>
+      </c>
+      <c r="L251" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_DERMATOLOGIC_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr"/>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Diabetic Foot Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>BOFAS / AOFAS Diabetic Foot Resources</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr"/>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G252" t="n">
+        <v>0</v>
+      </c>
+      <c r="H252" t="n">
+        <v>1</v>
+      </c>
+      <c r="I252" t="n">
+        <v>0</v>
+      </c>
+      <c r="J252" t="n">
+        <v>0</v>
+      </c>
+      <c r="K252" t="n">
+        <v>2</v>
+      </c>
+      <c r="L252" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_DIABETIC_FOOT_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Emergency General Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>society_page</t>
+        </is>
+      </c>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>AAST / WSES Emergency General Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr"/>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G253" t="n">
+        <v>0</v>
+      </c>
+      <c r="H253" t="n">
+        <v>1</v>
+      </c>
+      <c r="I253" t="n">
+        <v>0</v>
+      </c>
+      <c r="J253" t="n">
+        <v>0</v>
+      </c>
+      <c r="K253" t="n">
+        <v>2</v>
+      </c>
+      <c r="L253" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_EMERGENCY_GENERAL_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Endocrine Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>AAES / ESES Endocrine Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr"/>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G254" t="n">
+        <v>0</v>
+      </c>
+      <c r="H254" t="n">
+        <v>1</v>
+      </c>
+      <c r="I254" t="n">
+        <v>0</v>
+      </c>
+      <c r="J254" t="n">
+        <v>0</v>
+      </c>
+      <c r="K254" t="n">
+        <v>2</v>
+      </c>
+      <c r="L254" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_ENDOCRINE_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr"/>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>ENT Head and Neck Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>ENT UK / AHNS Head and Neck Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr"/>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G255" t="n">
+        <v>0</v>
+      </c>
+      <c r="H255" t="n">
+        <v>1</v>
+      </c>
+      <c r="I255" t="n">
+        <v>0</v>
+      </c>
+      <c r="J255" t="n">
+        <v>0</v>
+      </c>
+      <c r="K255" t="n">
+        <v>2</v>
+      </c>
+      <c r="L255" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_ENT_HEAD_NECK_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>B. Braun</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Epidural Kit</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>product_page</t>
+        </is>
+      </c>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>PERIFIX Continuous Epidural Set / Single Dose Epidural Tray</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr"/>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G256" t="n">
+        <v>1</v>
+      </c>
+      <c r="H256" t="n">
+        <v>3</v>
+      </c>
+      <c r="I256" t="n">
+        <v>2</v>
+      </c>
+      <c r="J256" t="n">
+        <v>0</v>
+      </c>
+      <c r="K256" t="n">
+        <v>0</v>
+      </c>
+      <c r="L256" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_EPIDURAL_KIT_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr"/>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Functional Neurosurgery Information System</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>CNS / WSSFN Functional Neurosurgery Resources</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr"/>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G257" t="n">
+        <v>0</v>
+      </c>
+      <c r="H257" t="n">
+        <v>1</v>
+      </c>
+      <c r="I257" t="n">
+        <v>0</v>
+      </c>
+      <c r="J257" t="n">
+        <v>0</v>
+      </c>
+      <c r="K257" t="n">
+        <v>2</v>
+      </c>
+      <c r="L257" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_FUNCTIONAL_NEUROSURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr"/>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Glaucoma Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>RCOphth / AGS Glaucoma Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr"/>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G258" t="n">
+        <v>0</v>
+      </c>
+      <c r="H258" t="n">
+        <v>1</v>
+      </c>
+      <c r="I258" t="n">
+        <v>0</v>
+      </c>
+      <c r="J258" t="n">
+        <v>0</v>
+      </c>
+      <c r="K258" t="n">
+        <v>2</v>
+      </c>
+      <c r="L258" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_GLAUCOMA_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr"/>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Gynecologic Oncology Information System</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>SGO / ESGO Gynecologic Oncology Resources</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr"/>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G259" t="n">
+        <v>0</v>
+      </c>
+      <c r="H259" t="n">
+        <v>1</v>
+      </c>
+      <c r="I259" t="n">
+        <v>0</v>
+      </c>
+      <c r="J259" t="n">
+        <v>0</v>
+      </c>
+      <c r="K259" t="n">
+        <v>2</v>
+      </c>
+      <c r="L259" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_GYNECOLOGIC_ONCOLOGY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr"/>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Gynecology Procedure Information System</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>BSGE / AAGL Gynecology Procedure Resources</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr"/>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G260" t="n">
+        <v>0</v>
+      </c>
+      <c r="H260" t="n">
+        <v>1</v>
+      </c>
+      <c r="I260" t="n">
+        <v>0</v>
+      </c>
+      <c r="J260" t="n">
+        <v>0</v>
+      </c>
+      <c r="K260" t="n">
+        <v>2</v>
+      </c>
+      <c r="L260" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_GYNECOLOGY_PROCEDURE_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr"/>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Hand and Microsurgery Information System</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>BAPRAS / BSSH Hand Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr"/>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G261" t="n">
+        <v>0</v>
+      </c>
+      <c r="H261" t="n">
+        <v>1</v>
+      </c>
+      <c r="I261" t="n">
+        <v>0</v>
+      </c>
+      <c r="J261" t="n">
+        <v>0</v>
+      </c>
+      <c r="K261" t="n">
+        <v>2</v>
+      </c>
+      <c r="L261" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_HAND_MICROSURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr"/>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Hernia Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>AHS / EHS Hernia Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr"/>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G262" t="n">
+        <v>0</v>
+      </c>
+      <c r="H262" t="n">
+        <v>1</v>
+      </c>
+      <c r="I262" t="n">
+        <v>0</v>
+      </c>
+      <c r="J262" t="n">
+        <v>0</v>
+      </c>
+      <c r="K262" t="n">
+        <v>2</v>
+      </c>
+      <c r="L262" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_HERNIA_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr"/>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>High Risk Obstetrics Information System</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>RCOG / SMFM High Risk Obstetrics Resources</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr"/>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G263" t="n">
+        <v>0</v>
+      </c>
+      <c r="H263" t="n">
+        <v>1</v>
+      </c>
+      <c r="I263" t="n">
+        <v>0</v>
+      </c>
+      <c r="J263" t="n">
+        <v>0</v>
+      </c>
+      <c r="K263" t="n">
+        <v>2</v>
+      </c>
+      <c r="L263" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_HIGH_RISK_OBSTETRICS_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>HPB Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>AHPBA / E-AHPBA HPB Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr"/>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G264" t="n">
+        <v>0</v>
+      </c>
+      <c r="H264" t="n">
+        <v>1</v>
+      </c>
+      <c r="I264" t="n">
+        <v>0</v>
+      </c>
+      <c r="J264" t="n">
+        <v>0</v>
+      </c>
+      <c r="K264" t="n">
+        <v>2</v>
+      </c>
+      <c r="L264" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_HPB_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>B. Braun</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Infusion Pump</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>product_page</t>
+        </is>
+      </c>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Infusomat Space Large Volume Pump</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr"/>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G265" t="n">
+        <v>0</v>
+      </c>
+      <c r="H265" t="n">
+        <v>3</v>
+      </c>
+      <c r="I265" t="n">
+        <v>2</v>
+      </c>
+      <c r="J265" t="n">
+        <v>0</v>
+      </c>
+      <c r="K265" t="n">
+        <v>1</v>
+      </c>
+      <c r="L265" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_INFUSION_PUMP_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr"/>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Laryngology and Airway Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>ENT UK / ELS Laryngology Resources</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr"/>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G266" t="n">
+        <v>0</v>
+      </c>
+      <c r="H266" t="n">
+        <v>1</v>
+      </c>
+      <c r="I266" t="n">
+        <v>0</v>
+      </c>
+      <c r="J266" t="n">
+        <v>0</v>
+      </c>
+      <c r="K266" t="n">
+        <v>2</v>
+      </c>
+      <c r="L266" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_LARYNGOLOGY_AIRWAY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr"/>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Maxillofacial Oncology and Reconstruction Information System</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D267" t="inlineStr">
+        <is>
+          <t>BAOMS / AAOMS Maxillofacial Oncology Resources</t>
+        </is>
+      </c>
+      <c r="E267" t="inlineStr"/>
+      <c r="F267" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G267" t="n">
+        <v>0</v>
+      </c>
+      <c r="H267" t="n">
+        <v>1</v>
+      </c>
+      <c r="I267" t="n">
+        <v>0</v>
+      </c>
+      <c r="J267" t="n">
+        <v>0</v>
+      </c>
+      <c r="K267" t="n">
+        <v>2</v>
+      </c>
+      <c r="L267" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_MAXILLOFACIAL_ONCOLOGY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr"/>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Maxillofacial Trauma Information System</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D268" t="inlineStr">
+        <is>
+          <t>BAOMS / AAOMS Maxillofacial Trauma Resources</t>
+        </is>
+      </c>
+      <c r="E268" t="inlineStr"/>
+      <c r="F268" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G268" t="n">
+        <v>0</v>
+      </c>
+      <c r="H268" t="n">
+        <v>1</v>
+      </c>
+      <c r="I268" t="n">
+        <v>0</v>
+      </c>
+      <c r="J268" t="n">
+        <v>0</v>
+      </c>
+      <c r="K268" t="n">
+        <v>2</v>
+      </c>
+      <c r="L268" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_MAXILLOFACIAL_TRAUMA_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr"/>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Minimally Invasive Gynecology Information System</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D269" t="inlineStr">
+        <is>
+          <t>BSGE / AAGL Minimally Invasive Gynecology Resources</t>
+        </is>
+      </c>
+      <c r="E269" t="inlineStr"/>
+      <c r="F269" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G269" t="n">
+        <v>0</v>
+      </c>
+      <c r="H269" t="n">
+        <v>1</v>
+      </c>
+      <c r="I269" t="n">
+        <v>0</v>
+      </c>
+      <c r="J269" t="n">
+        <v>0</v>
+      </c>
+      <c r="K269" t="n">
+        <v>2</v>
+      </c>
+      <c r="L269" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_MINIMALLY_INVASIVE_GYNECOLOGY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr"/>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Neonatal Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D270" t="inlineStr">
+        <is>
+          <t>BAPS / APSA Neonatal Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E270" t="inlineStr"/>
+      <c r="F270" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G270" t="n">
+        <v>0</v>
+      </c>
+      <c r="H270" t="n">
+        <v>1</v>
+      </c>
+      <c r="I270" t="n">
+        <v>0</v>
+      </c>
+      <c r="J270" t="n">
+        <v>0</v>
+      </c>
+      <c r="K270" t="n">
+        <v>2</v>
+      </c>
+      <c r="L270" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_NEONATAL_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>B. Braun</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Nerve Stimulator</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>product_page</t>
+        </is>
+      </c>
+      <c r="D271" t="inlineStr">
+        <is>
+          <t>Stimuplex HNS 12 Nerve Stimulator</t>
+        </is>
+      </c>
+      <c r="E271" t="inlineStr"/>
+      <c r="F271" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G271" t="n">
+        <v>0</v>
+      </c>
+      <c r="H271" t="n">
+        <v>3</v>
+      </c>
+      <c r="I271" t="n">
+        <v>3</v>
+      </c>
+      <c r="J271" t="n">
+        <v>0</v>
+      </c>
+      <c r="K271" t="n">
+        <v>1</v>
+      </c>
+      <c r="L271" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_NERVE_STIMULATOR_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr"/>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Neurooncology Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D272" t="inlineStr">
+        <is>
+          <t>CNS Tumor Section / EANO Neurooncology Resources</t>
+        </is>
+      </c>
+      <c r="E272" t="inlineStr"/>
+      <c r="F272" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G272" t="n">
+        <v>0</v>
+      </c>
+      <c r="H272" t="n">
+        <v>1</v>
+      </c>
+      <c r="I272" t="n">
+        <v>0</v>
+      </c>
+      <c r="J272" t="n">
+        <v>0</v>
+      </c>
+      <c r="K272" t="n">
+        <v>2</v>
+      </c>
+      <c r="L272" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_NEUROONCOLOGY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Obstetric Anaesthesia Workflow System</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D273" t="inlineStr">
+        <is>
+          <t>SOAP Society Resources / Educational App</t>
+        </is>
+      </c>
+      <c r="E273" t="inlineStr"/>
+      <c r="F273" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G273" t="n">
+        <v>0</v>
+      </c>
+      <c r="H273" t="n">
+        <v>1</v>
+      </c>
+      <c r="I273" t="n">
+        <v>0</v>
+      </c>
+      <c r="J273" t="n">
+        <v>0</v>
+      </c>
+      <c r="K273" t="n">
+        <v>2</v>
+      </c>
+      <c r="L273" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_OBSTETRIC_ANAESTHESIA_WORKFLOW_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr"/>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Oculoplastic Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D274" t="inlineStr">
+        <is>
+          <t>BOPSS / ASOPRS Oculoplastic Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E274" t="inlineStr"/>
+      <c r="F274" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G274" t="n">
+        <v>0</v>
+      </c>
+      <c r="H274" t="n">
+        <v>1</v>
+      </c>
+      <c r="I274" t="n">
+        <v>0</v>
+      </c>
+      <c r="J274" t="n">
+        <v>0</v>
+      </c>
+      <c r="K274" t="n">
+        <v>2</v>
+      </c>
+      <c r="L274" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_OCULOPLASTIC_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr"/>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Operative Delivery Information System</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D275" t="inlineStr">
+        <is>
+          <t>RCOG / ACOG Operative Delivery Resources</t>
+        </is>
+      </c>
+      <c r="E275" t="inlineStr"/>
+      <c r="F275" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G275" t="n">
+        <v>0</v>
+      </c>
+      <c r="H275" t="n">
+        <v>1</v>
+      </c>
+      <c r="I275" t="n">
+        <v>0</v>
+      </c>
+      <c r="J275" t="n">
+        <v>0</v>
+      </c>
+      <c r="K275" t="n">
+        <v>2</v>
+      </c>
+      <c r="L275" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_OPERATIVE_DELIVERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Oral Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>society_about_page</t>
+        </is>
+      </c>
+      <c r="D276" t="inlineStr">
+        <is>
+          <t>AAOMS / BAOMS Oral Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E276" t="inlineStr"/>
+      <c r="F276" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G276" t="n">
+        <v>0</v>
+      </c>
+      <c r="H276" t="n">
+        <v>1</v>
+      </c>
+      <c r="I276" t="n">
+        <v>0</v>
+      </c>
+      <c r="J276" t="n">
+        <v>0</v>
+      </c>
+      <c r="K276" t="n">
+        <v>2</v>
+      </c>
+      <c r="L276" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_ORAL_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr"/>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Orthofix Ankle arthroplasty Portfolio</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>portfolio_page</t>
+        </is>
+      </c>
+      <c r="D277" t="inlineStr">
+        <is>
+          <t>Orthofix Total Ankle Arthroplasty Portfolio</t>
+        </is>
+      </c>
+      <c r="E277" t="inlineStr"/>
+      <c r="F277" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G277" t="n">
+        <v>0</v>
+      </c>
+      <c r="H277" t="n">
+        <v>1</v>
+      </c>
+      <c r="I277" t="n">
+        <v>0</v>
+      </c>
+      <c r="J277" t="n">
+        <v>0</v>
+      </c>
+      <c r="K277" t="n">
+        <v>2</v>
+      </c>
+      <c r="L277" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_ORTHOFIX_ANKLE_ARTHROPLASTY_PORTFOLIO_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr"/>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Orthognathic Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D278" t="inlineStr">
+        <is>
+          <t>BAOMS / AAOMS Orthognathic Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E278" t="inlineStr"/>
+      <c r="F278" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G278" t="n">
+        <v>0</v>
+      </c>
+      <c r="H278" t="n">
+        <v>1</v>
+      </c>
+      <c r="I278" t="n">
+        <v>0</v>
+      </c>
+      <c r="J278" t="n">
+        <v>0</v>
+      </c>
+      <c r="K278" t="n">
+        <v>2</v>
+      </c>
+      <c r="L278" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_ORTHOGNATHIC_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr"/>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Otology and Neurotology Information System</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D279" t="inlineStr">
+        <is>
+          <t>ENT UK / EAONO Otology Resources</t>
+        </is>
+      </c>
+      <c r="E279" t="inlineStr"/>
+      <c r="F279" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G279" t="n">
+        <v>0</v>
+      </c>
+      <c r="H279" t="n">
+        <v>1</v>
+      </c>
+      <c r="I279" t="n">
+        <v>0</v>
+      </c>
+      <c r="J279" t="n">
+        <v>0</v>
+      </c>
+      <c r="K279" t="n">
+        <v>2</v>
+      </c>
+      <c r="L279" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_OTOLOGY_NEUROTOLOGY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Paediatric Anaesthesia Workflow System</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D280" t="inlineStr">
+        <is>
+          <t>Society for Pediatric Anesthesia / Resources</t>
+        </is>
+      </c>
+      <c r="E280" t="inlineStr"/>
+      <c r="F280" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G280" t="n">
+        <v>0</v>
+      </c>
+      <c r="H280" t="n">
+        <v>1</v>
+      </c>
+      <c r="I280" t="n">
+        <v>0</v>
+      </c>
+      <c r="J280" t="n">
+        <v>0</v>
+      </c>
+      <c r="K280" t="n">
+        <v>2</v>
+      </c>
+      <c r="L280" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_PAEDIATRIC_ANAESTHESIA_WORKFLOW_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr"/>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Paediatric Otolaryngology Information System</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D281" t="inlineStr">
+        <is>
+          <t>ENT UK / ESPO Paediatric ENT Resources</t>
+        </is>
+      </c>
+      <c r="E281" t="inlineStr"/>
+      <c r="F281" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G281" t="n">
+        <v>0</v>
+      </c>
+      <c r="H281" t="n">
+        <v>1</v>
+      </c>
+      <c r="I281" t="n">
+        <v>0</v>
+      </c>
+      <c r="J281" t="n">
+        <v>0</v>
+      </c>
+      <c r="K281" t="n">
+        <v>2</v>
+      </c>
+      <c r="L281" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_PAEDIATRIC_ENT_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr"/>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Paediatric General Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D282" t="inlineStr">
+        <is>
+          <t>BAPS / APSA Paediatric General Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E282" t="inlineStr"/>
+      <c r="F282" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G282" t="n">
+        <v>0</v>
+      </c>
+      <c r="H282" t="n">
+        <v>1</v>
+      </c>
+      <c r="I282" t="n">
+        <v>0</v>
+      </c>
+      <c r="J282" t="n">
+        <v>0</v>
+      </c>
+      <c r="K282" t="n">
+        <v>2</v>
+      </c>
+      <c r="L282" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_PAEDIATRIC_GENERAL_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr"/>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Paediatric Neurosurgery Information System</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D283" t="inlineStr">
+        <is>
+          <t>ISPN / ASPN Paediatric Neurosurgery Resources</t>
+        </is>
+      </c>
+      <c r="E283" t="inlineStr"/>
+      <c r="F283" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G283" t="n">
+        <v>0</v>
+      </c>
+      <c r="H283" t="n">
+        <v>1</v>
+      </c>
+      <c r="I283" t="n">
+        <v>0</v>
+      </c>
+      <c r="J283" t="n">
+        <v>0</v>
+      </c>
+      <c r="K283" t="n">
+        <v>2</v>
+      </c>
+      <c r="L283" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_PAEDIATRIC_NEUROSURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr"/>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Paediatric Ophthalmology Information System</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D284" t="inlineStr">
+        <is>
+          <t>RCOphth / AAPOS Paediatric Ophthalmology Resources</t>
+        </is>
+      </c>
+      <c r="E284" t="inlineStr"/>
+      <c r="F284" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G284" t="n">
+        <v>0</v>
+      </c>
+      <c r="H284" t="n">
+        <v>1</v>
+      </c>
+      <c r="I284" t="n">
+        <v>0</v>
+      </c>
+      <c r="J284" t="n">
+        <v>0</v>
+      </c>
+      <c r="K284" t="n">
+        <v>2</v>
+      </c>
+      <c r="L284" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_PAEDIATRIC_OPHTHALMOLOGY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr"/>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Paediatric Thoracic Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D285" t="inlineStr">
+        <is>
+          <t>BAPS / APSA Paediatric Thoracic Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E285" t="inlineStr"/>
+      <c r="F285" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G285" t="n">
+        <v>0</v>
+      </c>
+      <c r="H285" t="n">
+        <v>1</v>
+      </c>
+      <c r="I285" t="n">
+        <v>0</v>
+      </c>
+      <c r="J285" t="n">
+        <v>0</v>
+      </c>
+      <c r="K285" t="n">
+        <v>2</v>
+      </c>
+      <c r="L285" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_PAEDIATRIC_THORACIC_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr"/>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Paediatric Trauma Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D286" t="inlineStr">
+        <is>
+          <t>BAPS / APSA Paediatric Trauma Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E286" t="inlineStr"/>
+      <c r="F286" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G286" t="n">
+        <v>0</v>
+      </c>
+      <c r="H286" t="n">
+        <v>1</v>
+      </c>
+      <c r="I286" t="n">
+        <v>0</v>
+      </c>
+      <c r="J286" t="n">
+        <v>0</v>
+      </c>
+      <c r="K286" t="n">
+        <v>2</v>
+      </c>
+      <c r="L286" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_PAEDIATRIC_TRAUMA_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr"/>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Paragon 28 Ankle arthroplasty Portfolio</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>portfolio_page</t>
+        </is>
+      </c>
+      <c r="D287" t="inlineStr">
+        <is>
+          <t>Paragon 28 Ankle Arthroplasty Portfolio</t>
+        </is>
+      </c>
+      <c r="E287" t="inlineStr"/>
+      <c r="F287" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G287" t="n">
+        <v>0</v>
+      </c>
+      <c r="H287" t="n">
+        <v>1</v>
+      </c>
+      <c r="I287" t="n">
+        <v>0</v>
+      </c>
+      <c r="J287" t="n">
+        <v>0</v>
+      </c>
+      <c r="K287" t="n">
+        <v>2</v>
+      </c>
+      <c r="L287" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_PARAGON_28_ANKLE_ARTHROPLASTY_PORTFOLIO_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr"/>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Paragon 28 Total Ankle Portfolio</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>portfolio_page</t>
+        </is>
+      </c>
+      <c r="D288" t="inlineStr">
+        <is>
+          <t>Paragon 28 Total Ankle Portfolio</t>
+        </is>
+      </c>
+      <c r="E288" t="inlineStr"/>
+      <c r="F288" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G288" t="n">
+        <v>0</v>
+      </c>
+      <c r="H288" t="n">
+        <v>1</v>
+      </c>
+      <c r="I288" t="n">
+        <v>0</v>
+      </c>
+      <c r="J288" t="n">
+        <v>0</v>
+      </c>
+      <c r="K288" t="n">
+        <v>2</v>
+      </c>
+      <c r="L288" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_PARAGON_28_TOTAL_ANKLE_PORTFOLIO_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr"/>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Podiatric Forefoot Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D289" t="inlineStr">
+        <is>
+          <t>BOFAS / AOFAS Forefoot Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E289" t="inlineStr"/>
+      <c r="F289" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G289" t="n">
+        <v>0</v>
+      </c>
+      <c r="H289" t="n">
+        <v>1</v>
+      </c>
+      <c r="I289" t="n">
+        <v>0</v>
+      </c>
+      <c r="J289" t="n">
+        <v>0</v>
+      </c>
+      <c r="K289" t="n">
+        <v>2</v>
+      </c>
+      <c r="L289" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_PODIATRIC_FOREFOOT_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr"/>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Podiatric Midfoot Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D290" t="inlineStr">
+        <is>
+          <t>BOFAS / AOFAS Midfoot Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E290" t="inlineStr"/>
+      <c r="F290" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G290" t="n">
+        <v>0</v>
+      </c>
+      <c r="H290" t="n">
+        <v>1</v>
+      </c>
+      <c r="I290" t="n">
+        <v>0</v>
+      </c>
+      <c r="J290" t="n">
+        <v>0</v>
+      </c>
+      <c r="K290" t="n">
+        <v>2</v>
+      </c>
+      <c r="L290" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_PODIATRIC_MIDFOOT_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr"/>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Podiatric Rearfoot and Ankle Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D291" t="inlineStr">
+        <is>
+          <t>BOFAS / AOFAS Rearfoot and Ankle Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E291" t="inlineStr"/>
+      <c r="F291" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G291" t="n">
+        <v>0</v>
+      </c>
+      <c r="H291" t="n">
+        <v>1</v>
+      </c>
+      <c r="I291" t="n">
+        <v>0</v>
+      </c>
+      <c r="J291" t="n">
+        <v>0</v>
+      </c>
+      <c r="K291" t="n">
+        <v>2</v>
+      </c>
+      <c r="L291" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_PODIATRIC_REARFOOT_ANKLE_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Regional Anaesthesia Workflow System</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D292" t="inlineStr">
+        <is>
+          <t>ASRA / ESRA Regional Anaesthesia Resources</t>
+        </is>
+      </c>
+      <c r="E292" t="inlineStr"/>
+      <c r="F292" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G292" t="n">
+        <v>0</v>
+      </c>
+      <c r="H292" t="n">
+        <v>1</v>
+      </c>
+      <c r="I292" t="n">
+        <v>0</v>
+      </c>
+      <c r="J292" t="n">
+        <v>0</v>
+      </c>
+      <c r="K292" t="n">
+        <v>2</v>
+      </c>
+      <c r="L292" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_REGIONAL_ANAESTHESIA_WORKFLOW_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr"/>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Reproductive Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D293" t="inlineStr">
+        <is>
+          <t>ESHRE / ASRM Reproductive Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E293" t="inlineStr"/>
+      <c r="F293" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G293" t="n">
+        <v>0</v>
+      </c>
+      <c r="H293" t="n">
+        <v>1</v>
+      </c>
+      <c r="I293" t="n">
+        <v>0</v>
+      </c>
+      <c r="J293" t="n">
+        <v>0</v>
+      </c>
+      <c r="K293" t="n">
+        <v>2</v>
+      </c>
+      <c r="L293" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_REPRODUCTIVE_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr"/>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Rhinology and Sinus Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D294" t="inlineStr">
+        <is>
+          <t>ENT UK / ERS Rhinology Resources</t>
+        </is>
+      </c>
+      <c r="E294" t="inlineStr"/>
+      <c r="F294" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G294" t="n">
+        <v>0</v>
+      </c>
+      <c r="H294" t="n">
+        <v>1</v>
+      </c>
+      <c r="I294" t="n">
+        <v>0</v>
+      </c>
+      <c r="J294" t="n">
+        <v>0</v>
+      </c>
+      <c r="K294" t="n">
+        <v>2</v>
+      </c>
+      <c r="L294" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_RHINOLOGY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>Teleflex</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Supraglottic Airway Device</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>product_family_page</t>
+        </is>
+      </c>
+      <c r="D295" t="inlineStr">
+        <is>
+          <t>Supraglottic Airways | Teleflex</t>
+        </is>
+      </c>
+      <c r="E295" t="inlineStr"/>
+      <c r="F295" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G295" t="n">
+        <v>0</v>
+      </c>
+      <c r="H295" t="n">
+        <v>3</v>
+      </c>
+      <c r="I295" t="n">
+        <v>1</v>
+      </c>
+      <c r="J295" t="n">
+        <v>0</v>
+      </c>
+      <c r="K295" t="n">
+        <v>1</v>
+      </c>
+      <c r="L295" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_SGA_DEVICE_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr"/>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Smith+Nephew Hip revision arthroplasty Portfolio</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>portfolio_page</t>
+        </is>
+      </c>
+      <c r="D296" t="inlineStr">
+        <is>
+          <t>Smith+Nephew Revision Hip Arthroplasty Portfolio</t>
+        </is>
+      </c>
+      <c r="E296" t="inlineStr"/>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G296" t="n">
+        <v>0</v>
+      </c>
+      <c r="H296" t="n">
+        <v>1</v>
+      </c>
+      <c r="I296" t="n">
+        <v>0</v>
+      </c>
+      <c r="J296" t="n">
+        <v>0</v>
+      </c>
+      <c r="K296" t="n">
+        <v>2</v>
+      </c>
+      <c r="L296" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_SMITH_NEPHEW_HIP_REVISION_ARTHROPLASTY_PORTFOLIO_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>B. Braun</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Spinal Anaesthesia Kit</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>product_family_page</t>
+        </is>
+      </c>
+      <c r="D297" t="inlineStr">
+        <is>
+          <t>Spinocan / Pencan Spinal Anesthesia Trays</t>
+        </is>
+      </c>
+      <c r="E297" t="inlineStr"/>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G297" t="n">
+        <v>2</v>
+      </c>
+      <c r="H297" t="n">
+        <v>2</v>
+      </c>
+      <c r="I297" t="n">
+        <v>3</v>
+      </c>
+      <c r="J297" t="n">
+        <v>0</v>
+      </c>
+      <c r="K297" t="n">
+        <v>0</v>
+      </c>
+      <c r="L297" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_SPINAL_KIT_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr"/>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Spinal Neurosurgery Information System</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D298" t="inlineStr">
+        <is>
+          <t>CNS Spine Section / NASS Spinal Neurosurgery Resources</t>
+        </is>
+      </c>
+      <c r="E298" t="inlineStr"/>
+      <c r="F298" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G298" t="n">
+        <v>0</v>
+      </c>
+      <c r="H298" t="n">
+        <v>1</v>
+      </c>
+      <c r="I298" t="n">
+        <v>0</v>
+      </c>
+      <c r="J298" t="n">
+        <v>0</v>
+      </c>
+      <c r="K298" t="n">
+        <v>2</v>
+      </c>
+      <c r="L298" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_SPINAL_NEUROSURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr"/>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Stryker Elbow arthroplasty Portfolio</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>portfolio_page</t>
+        </is>
+      </c>
+      <c r="D299" t="inlineStr">
+        <is>
+          <t>Stryker Elbow Arthroplasty Portfolio</t>
+        </is>
+      </c>
+      <c r="E299" t="inlineStr"/>
+      <c r="F299" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G299" t="n">
+        <v>0</v>
+      </c>
+      <c r="H299" t="n">
+        <v>1</v>
+      </c>
+      <c r="I299" t="n">
+        <v>0</v>
+      </c>
+      <c r="J299" t="n">
+        <v>0</v>
+      </c>
+      <c r="K299" t="n">
+        <v>2</v>
+      </c>
+      <c r="L299" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_STRYKER_ELBOW_ARTHROPLASTY_PORTFOLIO_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr"/>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Stryker Elbow Revision Portfolio</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>portfolio_page</t>
+        </is>
+      </c>
+      <c r="D300" t="inlineStr">
+        <is>
+          <t>Stryker Elbow Revision Portfolio</t>
+        </is>
+      </c>
+      <c r="E300" t="inlineStr"/>
+      <c r="F300" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G300" t="n">
+        <v>0</v>
+      </c>
+      <c r="H300" t="n">
+        <v>1</v>
+      </c>
+      <c r="I300" t="n">
+        <v>0</v>
+      </c>
+      <c r="J300" t="n">
+        <v>0</v>
+      </c>
+      <c r="K300" t="n">
+        <v>2</v>
+      </c>
+      <c r="L300" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_STRYKER_ELBOW_REVISION_PORTFOLIO_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr"/>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Stryker Hip revision arthroplasty Portfolio</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>portfolio_page</t>
+        </is>
+      </c>
+      <c r="D301" t="inlineStr">
+        <is>
+          <t>Stryker Revision Hip Arthroplasty Portfolio</t>
+        </is>
+      </c>
+      <c r="E301" t="inlineStr"/>
+      <c r="F301" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G301" t="n">
+        <v>0</v>
+      </c>
+      <c r="H301" t="n">
+        <v>1</v>
+      </c>
+      <c r="I301" t="n">
+        <v>0</v>
+      </c>
+      <c r="J301" t="n">
+        <v>0</v>
+      </c>
+      <c r="K301" t="n">
+        <v>2</v>
+      </c>
+      <c r="L301" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_STRYKER_HIP_REVISION_ARTHROPLASTY_PORTFOLIO_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr"/>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Stryker Upper Extremity Arthroplasty Portfolio</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>portfolio_page</t>
+        </is>
+      </c>
+      <c r="D302" t="inlineStr">
+        <is>
+          <t>Stryker Upper Extremity Arthroplasty Portfolio</t>
+        </is>
+      </c>
+      <c r="E302" t="inlineStr"/>
+      <c r="F302" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G302" t="n">
+        <v>0</v>
+      </c>
+      <c r="H302" t="n">
+        <v>1</v>
+      </c>
+      <c r="I302" t="n">
+        <v>0</v>
+      </c>
+      <c r="J302" t="n">
+        <v>0</v>
+      </c>
+      <c r="K302" t="n">
+        <v>2</v>
+      </c>
+      <c r="L302" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_STRYKER_UPPER_EXTREMITY_ARTHROPLASTY_PORTFOLIO_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr"/>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Surgical Oncology Information System</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D303" t="inlineStr">
+        <is>
+          <t>SSO / ESSO Surgical Oncology Resources</t>
+        </is>
+      </c>
+      <c r="E303" t="inlineStr"/>
+      <c r="F303" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G303" t="n">
+        <v>0</v>
+      </c>
+      <c r="H303" t="n">
+        <v>1</v>
+      </c>
+      <c r="I303" t="n">
+        <v>0</v>
+      </c>
+      <c r="J303" t="n">
+        <v>0</v>
+      </c>
+      <c r="K303" t="n">
+        <v>2</v>
+      </c>
+      <c r="L303" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_SURGICAL_ONCOLOGY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Thoracic Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>society_about_page</t>
+        </is>
+      </c>
+      <c r="D304" t="inlineStr">
+        <is>
+          <t>STS / ESTS Thoracic Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E304" t="inlineStr"/>
+      <c r="F304" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G304" t="n">
+        <v>0</v>
+      </c>
+      <c r="H304" t="n">
+        <v>1</v>
+      </c>
+      <c r="I304" t="n">
+        <v>0</v>
+      </c>
+      <c r="J304" t="n">
+        <v>0</v>
+      </c>
+      <c r="K304" t="n">
+        <v>2</v>
+      </c>
+      <c r="L304" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_THORACIC_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr"/>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Temporomandibular Joint Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D305" t="inlineStr">
+        <is>
+          <t>BAOMS / AAOMS Temporomandibular Joint Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E305" t="inlineStr"/>
+      <c r="F305" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G305" t="n">
+        <v>0</v>
+      </c>
+      <c r="H305" t="n">
+        <v>1</v>
+      </c>
+      <c r="I305" t="n">
+        <v>0</v>
+      </c>
+      <c r="J305" t="n">
+        <v>0</v>
+      </c>
+      <c r="K305" t="n">
+        <v>2</v>
+      </c>
+      <c r="L305" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_TMJ_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr"/>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Transplant Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D306" t="inlineStr">
+        <is>
+          <t>ASTS / ESOT Transplant Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E306" t="inlineStr"/>
+      <c r="F306" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G306" t="n">
+        <v>0</v>
+      </c>
+      <c r="H306" t="n">
+        <v>1</v>
+      </c>
+      <c r="I306" t="n">
+        <v>0</v>
+      </c>
+      <c r="J306" t="n">
+        <v>0</v>
+      </c>
+      <c r="K306" t="n">
+        <v>2</v>
+      </c>
+      <c r="L306" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_TRANSPLANT_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>Fujifilm Medical</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Ultrasound Machine</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>product_family_page</t>
+        </is>
+      </c>
+      <c r="D307" t="inlineStr">
+        <is>
+          <t>Portable, Point-of-Care Ultrasound | FUJIFILM Sonosite</t>
+        </is>
+      </c>
+      <c r="E307" t="inlineStr"/>
+      <c r="F307" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G307" t="n">
+        <v>0</v>
+      </c>
+      <c r="H307" t="n">
+        <v>3</v>
+      </c>
+      <c r="I307" t="n">
+        <v>0</v>
+      </c>
+      <c r="J307" t="n">
+        <v>0</v>
+      </c>
+      <c r="K307" t="n">
+        <v>2</v>
+      </c>
+      <c r="L307" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_ULTRASOUND_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr"/>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Upper GI Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D308" t="inlineStr">
+        <is>
+          <t>AUGIS / ISDE Upper GI Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E308" t="inlineStr"/>
+      <c r="F308" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G308" t="n">
+        <v>0</v>
+      </c>
+      <c r="H308" t="n">
+        <v>1</v>
+      </c>
+      <c r="I308" t="n">
+        <v>0</v>
+      </c>
+      <c r="J308" t="n">
+        <v>0</v>
+      </c>
+      <c r="K308" t="n">
+        <v>2</v>
+      </c>
+      <c r="L308" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_UPPER_GI_SURGERY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr"/>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Urogynecology and Pelvic Floor Information System</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D309" t="inlineStr">
+        <is>
+          <t>IUGA / AUGS Urogynecology Resources</t>
+        </is>
+      </c>
+      <c r="E309" t="inlineStr"/>
+      <c r="F309" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G309" t="n">
+        <v>0</v>
+      </c>
+      <c r="H309" t="n">
+        <v>1</v>
+      </c>
+      <c r="I309" t="n">
+        <v>0</v>
+      </c>
+      <c r="J309" t="n">
+        <v>0</v>
+      </c>
+      <c r="K309" t="n">
+        <v>2</v>
+      </c>
+      <c r="L309" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_UROGYNECOLOGY_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr"/>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Vitreoretinal Surgery Information System</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>society_homepage</t>
+        </is>
+      </c>
+      <c r="D310" t="inlineStr">
+        <is>
+          <t>RCOphth / ASRS Vitreoretinal Surgery Resources</t>
+        </is>
+      </c>
+      <c r="E310" t="inlineStr"/>
+      <c r="F310" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G310" t="n">
+        <v>0</v>
+      </c>
+      <c r="H310" t="n">
+        <v>1</v>
+      </c>
+      <c r="I310" t="n">
+        <v>0</v>
+      </c>
+      <c r="J310" t="n">
+        <v>0</v>
+      </c>
+      <c r="K310" t="n">
+        <v>2</v>
+      </c>
+      <c r="L310" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_VITREORETINAL_INFORMATION_SYSTEM_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr"/>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Zimmer Biomet Acetabular Revision Portfolio</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>portfolio_page</t>
+        </is>
+      </c>
+      <c r="D311" t="inlineStr">
+        <is>
+          <t>Zimmer Biomet Revision Hip Portfolio</t>
+        </is>
+      </c>
+      <c r="E311" t="inlineStr"/>
+      <c r="F311" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G311" t="n">
+        <v>0</v>
+      </c>
+      <c r="H311" t="n">
+        <v>1</v>
+      </c>
+      <c r="I311" t="n">
+        <v>0</v>
+      </c>
+      <c r="J311" t="n">
+        <v>0</v>
+      </c>
+      <c r="K311" t="n">
+        <v>2</v>
+      </c>
+      <c r="L311" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_ZIMMER_BIOMET_ACETABULAR_REVISION_PORTFOLIO_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr"/>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Zimmer Biomet Ankle arthroplasty Portfolio</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>portfolio_page</t>
+        </is>
+      </c>
+      <c r="D312" t="inlineStr">
+        <is>
+          <t>Zimmer Biomet Ankle Arthroplasty Portfolio</t>
+        </is>
+      </c>
+      <c r="E312" t="inlineStr"/>
+      <c r="F312" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G312" t="n">
+        <v>0</v>
+      </c>
+      <c r="H312" t="n">
+        <v>1</v>
+      </c>
+      <c r="I312" t="n">
+        <v>0</v>
+      </c>
+      <c r="J312" t="n">
+        <v>0</v>
+      </c>
+      <c r="K312" t="n">
+        <v>2</v>
+      </c>
+      <c r="L312" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_ZIMMER_BIOMET_ANKLE_ARTHROPLASTY_PORTFOLIO_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr"/>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Zimmer Biomet Femoral Revision Portfolio</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>portfolio_page</t>
+        </is>
+      </c>
+      <c r="D313" t="inlineStr">
+        <is>
+          <t>Zimmer Biomet Revision Hip Portfolio</t>
+        </is>
+      </c>
+      <c r="E313" t="inlineStr"/>
+      <c r="F313" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="G313" t="n">
+        <v>0</v>
+      </c>
+      <c r="H313" t="n">
+        <v>1</v>
+      </c>
+      <c r="I313" t="n">
+        <v>0</v>
+      </c>
+      <c r="J313" t="n">
+        <v>0</v>
+      </c>
+      <c r="K313" t="n">
+        <v>2</v>
+      </c>
+      <c r="L313" t="inlineStr">
+        <is>
+          <t>data\catalogue\manual_extractions\2026-03-15\SYS_ZIMMER_BIOMET_FEMORAL_REVISION_PORTFOLIO_extraction.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr"/>
+      <c r="B314" t="inlineStr"/>
+      <c r="C314" t="inlineStr"/>
+      <c r="D314" t="inlineStr"/>
+      <c r="E314" t="inlineStr"/>
+      <c r="F314" t="inlineStr"/>
+      <c r="G314" t="n">
+        <v>0</v>
+      </c>
+      <c r="H314" t="n">
+        <v>0</v>
+      </c>
+      <c r="I314" t="n">
+        <v>0</v>
+      </c>
+      <c r="J314" t="n">
+        <v>0</v>
+      </c>
+      <c r="K314" t="n">
+        <v>0</v>
+      </c>
+      <c r="L314" t="inlineStr">
+        <is>
           <t>data\catalogue\manual_extractions\theatre-equipment\consumables_extraction.json</t>
         </is>
       </c>
     </row>
-    <row r="227">
-      <c r="A227" t="inlineStr"/>
-      <c r="B227" t="inlineStr"/>
-      <c r="C227" t="inlineStr"/>
-      <c r="D227" t="inlineStr"/>
-      <c r="E227" t="inlineStr"/>
-      <c r="F227" t="inlineStr"/>
-      <c r="G227" t="n">
-        <v>0</v>
-      </c>
-      <c r="H227" t="n">
-        <v>0</v>
-      </c>
-      <c r="I227" t="n">
-        <v>0</v>
-      </c>
-      <c r="J227" t="n">
-        <v>0</v>
-      </c>
-      <c r="K227" t="n">
-        <v>0</v>
-      </c>
-      <c r="L227" t="inlineStr">
+    <row r="315">
+      <c r="A315" t="inlineStr"/>
+      <c r="B315" t="inlineStr"/>
+      <c r="C315" t="inlineStr"/>
+      <c r="D315" t="inlineStr"/>
+      <c r="E315" t="inlineStr"/>
+      <c r="F315" t="inlineStr"/>
+      <c r="G315" t="n">
+        <v>0</v>
+      </c>
+      <c r="H315" t="n">
+        <v>0</v>
+      </c>
+      <c r="I315" t="n">
+        <v>0</v>
+      </c>
+      <c r="J315" t="n">
+        <v>0</v>
+      </c>
+      <c r="K315" t="n">
+        <v>0</v>
+      </c>
+      <c r="L315" t="inlineStr">
         <is>
           <t>data\catalogue\manual_extractions\theatre-equipment\operating_tables_extraction.json</t>
         </is>
       </c>
     </row>
-    <row r="228">
-      <c r="A228" t="inlineStr"/>
-      <c r="B228" t="inlineStr"/>
-      <c r="C228" t="inlineStr"/>
-      <c r="D228" t="inlineStr"/>
-      <c r="E228" t="inlineStr"/>
-      <c r="F228" t="inlineStr"/>
-      <c r="G228" t="n">
-        <v>0</v>
-      </c>
-      <c r="H228" t="n">
-        <v>0</v>
-      </c>
-      <c r="I228" t="n">
-        <v>0</v>
-      </c>
-      <c r="J228" t="n">
-        <v>0</v>
-      </c>
-      <c r="K228" t="n">
-        <v>0</v>
-      </c>
-      <c r="L228" t="inlineStr">
+    <row r="316">
+      <c r="A316" t="inlineStr"/>
+      <c r="B316" t="inlineStr"/>
+      <c r="C316" t="inlineStr"/>
+      <c r="D316" t="inlineStr"/>
+      <c r="E316" t="inlineStr"/>
+      <c r="F316" t="inlineStr"/>
+      <c r="G316" t="n">
+        <v>0</v>
+      </c>
+      <c r="H316" t="n">
+        <v>0</v>
+      </c>
+      <c r="I316" t="n">
+        <v>0</v>
+      </c>
+      <c r="J316" t="n">
+        <v>0</v>
+      </c>
+      <c r="K316" t="n">
+        <v>0</v>
+      </c>
+      <c r="L316" t="inlineStr">
         <is>
           <t>data\catalogue\manual_extractions\theatre-equipment\positioning_extraction.json</t>
         </is>
       </c>
     </row>
-    <row r="229">
-      <c r="A229" t="inlineStr"/>
-      <c r="B229" t="inlineStr"/>
-      <c r="C229" t="inlineStr"/>
-      <c r="D229" t="inlineStr"/>
-      <c r="E229" t="inlineStr"/>
-      <c r="F229" t="inlineStr"/>
-      <c r="G229" t="n">
-        <v>0</v>
-      </c>
-      <c r="H229" t="n">
-        <v>0</v>
-      </c>
-      <c r="I229" t="n">
-        <v>0</v>
-      </c>
-      <c r="J229" t="n">
-        <v>0</v>
-      </c>
-      <c r="K229" t="n">
-        <v>0</v>
-      </c>
-      <c r="L229" t="inlineStr">
+    <row r="317">
+      <c r="A317" t="inlineStr"/>
+      <c r="B317" t="inlineStr"/>
+      <c r="C317" t="inlineStr"/>
+      <c r="D317" t="inlineStr"/>
+      <c r="E317" t="inlineStr"/>
+      <c r="F317" t="inlineStr"/>
+      <c r="G317" t="n">
+        <v>0</v>
+      </c>
+      <c r="H317" t="n">
+        <v>0</v>
+      </c>
+      <c r="I317" t="n">
+        <v>0</v>
+      </c>
+      <c r="J317" t="n">
+        <v>0</v>
+      </c>
+      <c r="K317" t="n">
+        <v>0</v>
+      </c>
+      <c r="L317" t="inlineStr">
         <is>
           <t>data\catalogue\manual_extractions\theatre-equipment\theatre_equipment_extraction.json</t>
         </is>

</xml_diff>